<commit_message>
Added Latest DataBase Export and Excel Export
</commit_message>
<xml_diff>
--- a/03_Learning_Management/00_Excel_Export/videos.xlsx
+++ b/03_Learning_Management/00_Excel_Export/videos.xlsx
@@ -433,16 +433,16 @@
         <v>101</v>
       </c>
       <c r="C2" t="str">
-        <v>Communication Skill</v>
+        <v>English</v>
       </c>
       <c r="D2" t="str">
-        <v>बोलने में माहिर कैसे बनें? | Think Fast, Talk Smart : Communication Techniques | Hindi Audiobook</v>
+        <v>How to Use Was, Did &amp; Had in Real English Conversations</v>
       </c>
       <c r="E2" t="str">
-        <v>Rethink and Legend Biography</v>
+        <v>English Daily Practice</v>
       </c>
       <c r="F2" t="str">
-        <v>https://www.youtube.com/watch?v=buJTqUIKMdQ</v>
+        <v>https://www.youtube.com/watch?v=oP5XXkp7W_E</v>
       </c>
       <c r="G2" t="str">
         <v>No</v>
@@ -459,19 +459,19 @@
         <v>101</v>
       </c>
       <c r="C3" t="str">
-        <v>Communication Skill</v>
+        <v>English</v>
       </c>
       <c r="D3" t="str">
-        <v>Episode 1: How To Master Communication Skills | Communication Mastery Series by Aakash Gupta</v>
+        <v>Learn ENGLISH with ChatGPT in 100 Days - 4 Step Method! | Warikoo Careers Hindi</v>
       </c>
       <c r="E3" t="str">
-        <v>Aakash Guptaa</v>
+        <v>Warikoo Careers</v>
       </c>
       <c r="F3" t="str">
-        <v>https://www.youtube.com/watch?v=hJegA740NEo&amp;list=PLv9O1ieIsEgfbNVwPqWxlZq_JtKmnsubv</v>
+        <v>https://www.youtube.com/watch?v=sHpgX2FnToM</v>
       </c>
       <c r="G3" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
       <c r="H3" t="str">
         <v>No</v>
@@ -485,16 +485,16 @@
         <v>101</v>
       </c>
       <c r="C4" t="str">
-        <v>Communication Skill</v>
+        <v>English</v>
       </c>
       <c r="D4" t="str">
-        <v>Interview Questions and Answers! (How to PASS a JOB INTERVIEW!)</v>
+        <v>English Podcast for Beginners - How to Think in English | Stop Translating in Your Head Now</v>
       </c>
       <c r="E4" t="str">
-        <v>CareerVidz</v>
+        <v>Mr. English Channel</v>
       </c>
       <c r="F4" t="str">
-        <v>https://www.youtube.com/watch?v=KCm6JVtoRdo</v>
+        <v>https://www.youtube.com/watch?v=uv9o385wyZ8</v>
       </c>
       <c r="G4" t="str">
         <v>No</v>
@@ -511,16 +511,16 @@
         <v>101</v>
       </c>
       <c r="C5" t="str">
-        <v>Communication Skill</v>
+        <v>English</v>
       </c>
       <c r="D5" t="str">
-        <v>If You Know These 36 Words, Your English is EXCELLENT!</v>
+        <v>Don't Act Weird Next Time You Hear Them!</v>
       </c>
       <c r="E5" t="str">
-        <v>Aleena Rais Live</v>
+        <v>Filmglish Academy</v>
       </c>
       <c r="F5" t="str">
-        <v>https://www.youtube.com/watch?v=7AW6ORQLWvU</v>
+        <v>https://www.youtube.com/watch?v=wVQ5R6Te1Ik</v>
       </c>
       <c r="G5" t="str">
         <v>No</v>
@@ -537,16 +537,16 @@
         <v>101</v>
       </c>
       <c r="C6" t="str">
-        <v>Communication Skill</v>
+        <v>English</v>
       </c>
       <c r="D6" t="str">
-        <v>How to Quickly Articulate a Response to Any Question - Priyanka Chopra’s SECRET is OUT</v>
+        <v>🎤 How to Train Your Brain to Speak English Fluently || Boost Your English Speaking Skills</v>
       </c>
       <c r="E6" t="str">
-        <v>Aleena Rais Live</v>
+        <v>Next Level Motivation</v>
       </c>
       <c r="F6" t="str">
-        <v>https://www.youtube.com/watch?v=wkFkWdGiLrQ</v>
+        <v>https://www.youtube.com/watch?v=_wqeFA0qrQo</v>
       </c>
       <c r="G6" t="str">
         <v>No</v>
@@ -563,16 +563,16 @@
         <v>101</v>
       </c>
       <c r="C7" t="str">
-        <v>Communication Skill</v>
+        <v>English</v>
       </c>
       <c r="D7" t="str">
-        <v>Watch This Before Your Next Interview !</v>
+        <v>Band 9 IELTS Speaking interview (Perfect Pronunciation)</v>
       </c>
       <c r="E7" t="str">
-        <v>Freshers GPT</v>
+        <v>BARC TV</v>
       </c>
       <c r="F7" t="str">
-        <v>https://www.youtube.com/watch?v=EGf7w7skQ_Q</v>
+        <v>https://www.youtube.com/watch?v=Mr2f4MxGmA8</v>
       </c>
       <c r="G7" t="str">
         <v>No</v>
@@ -589,16 +589,16 @@
         <v>101</v>
       </c>
       <c r="C8" t="str">
-        <v>Communication Skill</v>
+        <v>English</v>
       </c>
       <c r="D8" t="str">
-        <v>Why You Can't Communicate Properly (And How to Fix It) !</v>
+        <v>The Roadmap That Made Me Fluent in English (Fast &amp; Alone)</v>
       </c>
       <c r="E8" t="str">
-        <v>Freshers GPT</v>
+        <v>Joao Sales</v>
       </c>
       <c r="F8" t="str">
-        <v>https://www.youtube.com/watch?v=M0Is1-c5wDs</v>
+        <v>https://www.youtube.com/watch?v=FIhqFYAr0sM</v>
       </c>
       <c r="G8" t="str">
         <v>No</v>
@@ -615,16 +615,16 @@
         <v>101</v>
       </c>
       <c r="C9" t="str">
-        <v>Communication Skill</v>
+        <v>English</v>
       </c>
       <c r="D9" t="str">
-        <v>Struggling with English? What Finally Worked for Me to Speak Confidently!</v>
+        <v>How To Manage Your Time | English Podcast For Easy English Conversation | Don’t Waste Your Life</v>
       </c>
       <c r="E9" t="str">
-        <v>Thasaanthan</v>
+        <v>Speak English With Class</v>
       </c>
       <c r="F9" t="str">
-        <v>https://www.youtube.com/watch?v=6XlvBpRl418</v>
+        <v>https://www.youtube.com/watch?v=wRoz020CqOs</v>
       </c>
       <c r="G9" t="str">
         <v>No</v>
@@ -641,16 +641,16 @@
         <v>101</v>
       </c>
       <c r="C10" t="str">
-        <v>Communication Skill</v>
+        <v>English</v>
       </c>
       <c r="D10" t="str">
-        <v>English Communication Playlist</v>
+        <v>Day 3 | How Good Is Your English? Take This Test Before You Continue | English Speaking Course</v>
       </c>
       <c r="E10" t="str">
-        <v>Awal Creations</v>
+        <v>Ocean English Academy</v>
       </c>
       <c r="F10" t="str">
-        <v>https://www.youtube.com/@awalcreations/playlists</v>
+        <v>https://www.youtube.com/watch?v=s6eBVmvL6no</v>
       </c>
       <c r="G10" t="str">
         <v>No</v>
@@ -667,16 +667,16 @@
         <v>101</v>
       </c>
       <c r="C11" t="str">
-        <v>Communication Skill</v>
+        <v>English</v>
       </c>
       <c r="D11" t="str">
-        <v>The Only Video You Need To Fix Your Communication Skills</v>
+        <v>This Simple Habit Will Make You Fluent in English (backed by science)</v>
       </c>
       <c r="E11" t="str">
-        <v>Vinh Giang</v>
+        <v>Veronika's Language Diaries</v>
       </c>
       <c r="F11" t="str">
-        <v>https://www.youtube.com/watch?v=HlY0Awdpf9U</v>
+        <v>https://www.youtube.com/watch?v=f96t2rsb4Lw</v>
       </c>
       <c r="G11" t="str">
         <v>No</v>
@@ -693,16 +693,16 @@
         <v>101</v>
       </c>
       <c r="C12" t="str">
-        <v>Communication Skill</v>
+        <v>English</v>
       </c>
       <c r="D12" t="str">
-        <v>9 Habits for Clearer Speaking (I Wish I Knew Sooner)</v>
+        <v>Talking About Awkward Situations in English | Easy English Podcast</v>
       </c>
       <c r="E12" t="str">
-        <v>Vinh Giang</v>
+        <v>Everyday English Academy</v>
       </c>
       <c r="F12" t="str">
-        <v>https://www.youtube.com/watch?v=PiNN-HmHu7A</v>
+        <v>https://www.youtube.com/watch?v=eN6u3m3OFjI</v>
       </c>
       <c r="G12" t="str">
         <v>No</v>
@@ -719,16 +719,16 @@
         <v>101</v>
       </c>
       <c r="C13" t="str">
-        <v>Communication Skill</v>
+        <v>English</v>
       </c>
       <c r="D13" t="str">
-        <v>Understand English But Can’t Speak? Fix It Now!</v>
+        <v>How to build English Sentences</v>
       </c>
       <c r="E13" t="str">
-        <v>POC English</v>
+        <v>The English Class</v>
       </c>
       <c r="F13" t="str">
-        <v>https://www.youtube.com/watch?v=kawR96Gi6Xo</v>
+        <v>https://www.youtube.com/watch?v=hJ7PzBD9a2g</v>
       </c>
       <c r="G13" t="str">
         <v>No</v>
@@ -745,16 +745,16 @@
         <v>101</v>
       </c>
       <c r="C14" t="str">
-        <v>Communication Skill</v>
+        <v>English</v>
       </c>
       <c r="D14" t="str">
-        <v>How to Build Confidence &amp; Rule the World 🏆</v>
+        <v>How to Understand English Movies Without Subtitles</v>
       </c>
       <c r="E14" t="str">
-        <v>Riya Upreti</v>
+        <v>The English Class</v>
       </c>
       <c r="F14" t="str">
-        <v>https://www.youtube.com/watch?v=G05dmSjMoCU</v>
+        <v>https://www.youtube.com/watch?v=tB88DEBk5tw</v>
       </c>
       <c r="G14" t="str">
         <v>No</v>
@@ -771,16 +771,16 @@
         <v>101</v>
       </c>
       <c r="C15" t="str">
-        <v>Communication Skill</v>
+        <v>English</v>
       </c>
       <c r="D15" t="str">
-        <v>Why your English is BETTER than you think</v>
+        <v>Improve Your English Speaking Skills with Shadowing Practice | English Speaking Practice Podcast</v>
       </c>
       <c r="E15" t="str">
-        <v>English At the Ready</v>
+        <v>English In Minutes</v>
       </c>
       <c r="F15" t="str">
-        <v>https://www.youtube.com/watch?v=qoN70QgC-xI</v>
+        <v>https://www.youtube.com/watch?v=CSZOz5M_ztM</v>
       </c>
       <c r="G15" t="str">
         <v>No</v>
@@ -797,16 +797,16 @@
         <v>101</v>
       </c>
       <c r="C16" t="str">
-        <v>Communication Skill</v>
+        <v>English</v>
       </c>
       <c r="D16" t="str">
-        <v>🔥 1000 रोज़ बोले जाने वाले Words || Most Important English Words || Daily Use Word Meaning Practice</v>
+        <v>How to Speak English Without Thinking? | English Listening Practice | English Podcast</v>
       </c>
       <c r="E16" t="str">
-        <v>English ka Gurukul</v>
+        <v>English Hoot</v>
       </c>
       <c r="F16" t="str">
-        <v>https://www.youtube.com/watch?v=qoc3d33t3sY</v>
+        <v>https://www.youtube.com/watch?v=QSmEk7qcNNo</v>
       </c>
       <c r="G16" t="str">
         <v>No</v>
@@ -823,16 +823,16 @@
         <v>101</v>
       </c>
       <c r="C17" t="str">
-        <v>Communication Skill</v>
+        <v>English</v>
       </c>
       <c r="D17" t="str">
-        <v>How to THINK in English (and why you must)</v>
+        <v>ChatGPT for English Learners | Learn English | Chatgpt | Chat gpt | How To Learn Chatgpt | Viral</v>
       </c>
       <c r="E17" t="str">
-        <v>English At the Ready</v>
+        <v>English Titans</v>
       </c>
       <c r="F17" t="str">
-        <v>https://www.youtube.com/watch?v=cohlqUEtFXs</v>
+        <v>https://www.youtube.com/watch?v=domNltlQCxc</v>
       </c>
       <c r="G17" t="str">
         <v>No</v>
@@ -849,16 +849,16 @@
         <v>101</v>
       </c>
       <c r="C18" t="str">
-        <v>Communication Skill</v>
+        <v>English</v>
       </c>
       <c r="D18" t="str">
-        <v>How To Speak English With Just 521 Words | No Grammar, No Difficult Words, No Teacher, No Long Time</v>
+        <v>Advance English Structure | Daily Use English Sentence in Spoken English | English Speaking Practice</v>
       </c>
       <c r="E18" t="str">
-        <v>Easy English:The PodCast</v>
+        <v>Daily English With Sony</v>
       </c>
       <c r="F18" t="str">
-        <v>https://www.youtube.com/watch?v=ilHfpmbP0h8</v>
+        <v>https://www.youtube.com/watch?v=0G9RWEGT60Y</v>
       </c>
       <c r="G18" t="str">
         <v>No</v>
@@ -872,19 +872,19 @@
         <v>General</v>
       </c>
       <c r="B19">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="C19" t="str">
         <v>English</v>
       </c>
       <c r="D19" t="str">
-        <v>The Roadmap That Made Me Fluent in English (Fast &amp; Alone)</v>
+        <v>Watch this and everyone will think you're a native English speaker!</v>
       </c>
       <c r="E19" t="str">
-        <v>Joao Sales</v>
+        <v>Real English From Movies</v>
       </c>
       <c r="F19" t="str">
-        <v>https://www.youtube.com/watch?v=FIhqFYAr0sM</v>
+        <v>https://www.youtube.com/watch?v=OaDhB9tgBUE</v>
       </c>
       <c r="G19" t="str">
         <v>No</v>
@@ -898,19 +898,19 @@
         <v>General</v>
       </c>
       <c r="B20">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="C20" t="str">
         <v>English</v>
       </c>
       <c r="D20" t="str">
-        <v>Learn ENGLISH with ChatGPT in 100 Days - 4 Step Method! | Warikoo Careers Hindi</v>
+        <v>Watch this and you'll finally speak English like in the movies! 🎬</v>
       </c>
       <c r="E20" t="str">
-        <v>Warikoo Careers</v>
+        <v>Real English From Movies</v>
       </c>
       <c r="F20" t="str">
-        <v>https://www.youtube.com/watch?v=sHpgX2FnToM</v>
+        <v>https://www.youtube.com/watch?v=xHkHOfdp4FA</v>
       </c>
       <c r="G20" t="str">
         <v>No</v>
@@ -924,19 +924,19 @@
         <v>General</v>
       </c>
       <c r="B21">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="C21" t="str">
         <v>English</v>
       </c>
       <c r="D21" t="str">
-        <v>English Podcast for Beginners - How to Think in English | Stop Translating in Your Head Now</v>
+        <v>Learn All Modal Auxiliary Verb | modal verbs in english | Modal Verbs #prienglishclasses</v>
       </c>
       <c r="E21" t="str">
-        <v>Mr. English Channel</v>
+        <v>PRi English Classes</v>
       </c>
       <c r="F21" t="str">
-        <v>https://www.youtube.com/watch?v=uv9o385wyZ8</v>
+        <v>https://www.youtube.com/watch?v=75YfMDuRmLw</v>
       </c>
       <c r="G21" t="str">
         <v>No</v>
@@ -950,19 +950,19 @@
         <v>General</v>
       </c>
       <c r="B22">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="C22" t="str">
         <v>English</v>
       </c>
       <c r="D22" t="str">
-        <v>Don't Act Weird Next Time You Hear Them!</v>
+        <v>90 days Plan to Speak English Confidently | Janhavi Panwar</v>
       </c>
       <c r="E22" t="str">
-        <v>Filmglish Academy</v>
+        <v>Janhavi Panwar</v>
       </c>
       <c r="F22" t="str">
-        <v>https://www.youtube.com/watch?v=wVQ5R6Te1Ik</v>
+        <v>https://www.youtube.com/watch?v=9T54hO6h1us</v>
       </c>
       <c r="G22" t="str">
         <v>No</v>
@@ -979,16 +979,16 @@
         <v>102</v>
       </c>
       <c r="C23" t="str">
-        <v>English</v>
+        <v>Communication Skill</v>
       </c>
       <c r="D23" t="str">
-        <v>🎤 How to Train Your Brain to Speak English Fluently || Boost Your English Speaking Skills</v>
+        <v>How To Speak English With Just 521 Words | No Grammar, No Difficult Words, No Teacher, No Long Time</v>
       </c>
       <c r="E23" t="str">
-        <v>Next Level Motivation</v>
+        <v>Easy English:The PodCast</v>
       </c>
       <c r="F23" t="str">
-        <v>https://www.youtube.com/watch?v=_wqeFA0qrQo</v>
+        <v>https://www.youtube.com/watch?v=ilHfpmbP0h8</v>
       </c>
       <c r="G23" t="str">
         <v>No</v>
@@ -1005,16 +1005,16 @@
         <v>102</v>
       </c>
       <c r="C24" t="str">
-        <v>English</v>
+        <v>Communication Skill</v>
       </c>
       <c r="D24" t="str">
-        <v>Band 9 IELTS Speaking interview (Perfect Pronunciation)</v>
+        <v>Understand English But Can’t Speak? Fix It Now!</v>
       </c>
       <c r="E24" t="str">
-        <v>BARC TV</v>
+        <v>POC English</v>
       </c>
       <c r="F24" t="str">
-        <v>https://www.youtube.com/watch?v=Mr2f4MxGmA8</v>
+        <v>https://www.youtube.com/watch?v=kawR96Gi6Xo</v>
       </c>
       <c r="G24" t="str">
         <v>No</v>
@@ -1031,19 +1031,19 @@
         <v>102</v>
       </c>
       <c r="C25" t="str">
-        <v>English</v>
+        <v>Communication Skill</v>
       </c>
       <c r="D25" t="str">
-        <v>How To Manage Your Time | English Podcast For Easy English Conversation | Don’t Waste Your Life</v>
+        <v>Episode 1: How To Master Communication Skills | Communication Mastery Series by Aakash Gupta</v>
       </c>
       <c r="E25" t="str">
-        <v>Speak English With Class</v>
+        <v>Aakash Guptaa</v>
       </c>
       <c r="F25" t="str">
-        <v>https://www.youtube.com/watch?v=wRoz020CqOs</v>
+        <v>https://www.youtube.com/watch?v=hJegA740NEo&amp;list=PLv9O1ieIsEgfbNVwPqWxlZq_JtKmnsubv</v>
       </c>
       <c r="G25" t="str">
-        <v>No</v>
+        <v>Yes</v>
       </c>
       <c r="H25" t="str">
         <v>No</v>
@@ -1057,16 +1057,16 @@
         <v>102</v>
       </c>
       <c r="C26" t="str">
-        <v>English</v>
+        <v>Communication Skill</v>
       </c>
       <c r="D26" t="str">
-        <v>Day 3 | How Good Is Your English? Take This Test Before You Continue | English Speaking Course</v>
+        <v>Interview Questions and Answers! (How to PASS a JOB INTERVIEW!)</v>
       </c>
       <c r="E26" t="str">
-        <v>Ocean English Academy</v>
+        <v>CareerVidz</v>
       </c>
       <c r="F26" t="str">
-        <v>https://www.youtube.com/watch?v=s6eBVmvL6no</v>
+        <v>https://www.youtube.com/watch?v=KCm6JVtoRdo</v>
       </c>
       <c r="G26" t="str">
         <v>No</v>
@@ -1083,16 +1083,16 @@
         <v>102</v>
       </c>
       <c r="C27" t="str">
-        <v>English</v>
+        <v>Communication Skill</v>
       </c>
       <c r="D27" t="str">
-        <v>This Simple Habit Will Make You Fluent in English (backed by science)</v>
+        <v>If You Know These 36 Words, Your English is EXCELLENT!</v>
       </c>
       <c r="E27" t="str">
-        <v>Veronika's Language Diaries</v>
+        <v>Aleena Rais Live</v>
       </c>
       <c r="F27" t="str">
-        <v>https://www.youtube.com/watch?v=f96t2rsb4Lw</v>
+        <v>https://www.youtube.com/watch?v=7AW6ORQLWvU</v>
       </c>
       <c r="G27" t="str">
         <v>No</v>
@@ -1109,16 +1109,16 @@
         <v>102</v>
       </c>
       <c r="C28" t="str">
-        <v>English</v>
+        <v>Communication Skill</v>
       </c>
       <c r="D28" t="str">
-        <v>Talking About Awkward Situations in English | Easy English Podcast</v>
+        <v>How to Quickly Articulate a Response to Any Question - Priyanka Chopra’s SECRET is OUT</v>
       </c>
       <c r="E28" t="str">
-        <v>Everyday English Academy</v>
+        <v>Aleena Rais Live</v>
       </c>
       <c r="F28" t="str">
-        <v>https://www.youtube.com/watch?v=eN6u3m3OFjI</v>
+        <v>https://www.youtube.com/watch?v=wkFkWdGiLrQ</v>
       </c>
       <c r="G28" t="str">
         <v>No</v>
@@ -1135,16 +1135,16 @@
         <v>102</v>
       </c>
       <c r="C29" t="str">
-        <v>English</v>
+        <v>Communication Skill</v>
       </c>
       <c r="D29" t="str">
-        <v>How to Use Was, Did &amp; Had in Real English Conversations</v>
+        <v>बोलने में माहिर कैसे बनें? | Think Fast, Talk Smart : Communication Techniques | Hindi Audiobook</v>
       </c>
       <c r="E29" t="str">
-        <v>English Daily Practice</v>
+        <v>Rethink and Legend Biography</v>
       </c>
       <c r="F29" t="str">
-        <v>https://www.youtube.com/watch?v=oP5XXkp7W_E</v>
+        <v>https://www.youtube.com/watch?v=buJTqUIKMdQ</v>
       </c>
       <c r="G29" t="str">
         <v>No</v>
@@ -1161,16 +1161,16 @@
         <v>102</v>
       </c>
       <c r="C30" t="str">
-        <v>English</v>
+        <v>Communication Skill</v>
       </c>
       <c r="D30" t="str">
-        <v>How to build English Sentences</v>
+        <v>Watch This Before Your Next Interview !</v>
       </c>
       <c r="E30" t="str">
-        <v>The English Class</v>
+        <v>Freshers GPT</v>
       </c>
       <c r="F30" t="str">
-        <v>https://www.youtube.com/watch?v=hJ7PzBD9a2g</v>
+        <v>https://www.youtube.com/watch?v=EGf7w7skQ_Q</v>
       </c>
       <c r="G30" t="str">
         <v>No</v>
@@ -1187,16 +1187,16 @@
         <v>102</v>
       </c>
       <c r="C31" t="str">
-        <v>English</v>
+        <v>Communication Skill</v>
       </c>
       <c r="D31" t="str">
-        <v>How to Understand English Movies Without Subtitles</v>
+        <v>Why You Can't Communicate Properly (And How to Fix It) !</v>
       </c>
       <c r="E31" t="str">
-        <v>The English Class</v>
+        <v>Freshers GPT</v>
       </c>
       <c r="F31" t="str">
-        <v>https://www.youtube.com/watch?v=tB88DEBk5tw</v>
+        <v>https://www.youtube.com/watch?v=M0Is1-c5wDs</v>
       </c>
       <c r="G31" t="str">
         <v>No</v>
@@ -1213,16 +1213,16 @@
         <v>102</v>
       </c>
       <c r="C32" t="str">
-        <v>English</v>
+        <v>Communication Skill</v>
       </c>
       <c r="D32" t="str">
-        <v>Improve Your English Speaking Skills with Shadowing Practice | English Speaking Practice Podcast</v>
+        <v>Struggling with English? What Finally Worked for Me to Speak Confidently!</v>
       </c>
       <c r="E32" t="str">
-        <v>English In Minutes</v>
+        <v>Thasaanthan</v>
       </c>
       <c r="F32" t="str">
-        <v>https://www.youtube.com/watch?v=CSZOz5M_ztM</v>
+        <v>https://www.youtube.com/watch?v=6XlvBpRl418</v>
       </c>
       <c r="G32" t="str">
         <v>No</v>
@@ -1239,16 +1239,16 @@
         <v>102</v>
       </c>
       <c r="C33" t="str">
-        <v>English</v>
+        <v>Communication Skill</v>
       </c>
       <c r="D33" t="str">
-        <v>How to Speak English Without Thinking? | English Listening Practice | English Podcast</v>
+        <v>English Communication Playlist</v>
       </c>
       <c r="E33" t="str">
-        <v>English Hoot</v>
+        <v>Awal Creations</v>
       </c>
       <c r="F33" t="str">
-        <v>https://www.youtube.com/watch?v=QSmEk7qcNNo</v>
+        <v>https://www.youtube.com/@awalcreations/playlists</v>
       </c>
       <c r="G33" t="str">
         <v>No</v>
@@ -1265,16 +1265,16 @@
         <v>102</v>
       </c>
       <c r="C34" t="str">
-        <v>English</v>
+        <v>Communication Skill</v>
       </c>
       <c r="D34" t="str">
-        <v>ChatGPT for English Learners | Learn English | Chatgpt | Chat gpt | How To Learn Chatgpt | Viral</v>
+        <v>The Only Video You Need To Fix Your Communication Skills</v>
       </c>
       <c r="E34" t="str">
-        <v>English Titans</v>
+        <v>Vinh Giang</v>
       </c>
       <c r="F34" t="str">
-        <v>https://www.youtube.com/watch?v=domNltlQCxc</v>
+        <v>https://www.youtube.com/watch?v=HlY0Awdpf9U</v>
       </c>
       <c r="G34" t="str">
         <v>No</v>
@@ -1291,16 +1291,16 @@
         <v>102</v>
       </c>
       <c r="C35" t="str">
-        <v>English</v>
+        <v>Communication Skill</v>
       </c>
       <c r="D35" t="str">
-        <v>Advance English Structure | Daily Use English Sentence in Spoken English | English Speaking Practice</v>
+        <v>9 Habits for Clearer Speaking (I Wish I Knew Sooner)</v>
       </c>
       <c r="E35" t="str">
-        <v>Daily English With Sony</v>
+        <v>Vinh Giang</v>
       </c>
       <c r="F35" t="str">
-        <v>https://www.youtube.com/watch?v=0G9RWEGT60Y</v>
+        <v>https://www.youtube.com/watch?v=PiNN-HmHu7A</v>
       </c>
       <c r="G35" t="str">
         <v>No</v>
@@ -1317,16 +1317,16 @@
         <v>102</v>
       </c>
       <c r="C36" t="str">
-        <v>English</v>
+        <v>Communication Skill</v>
       </c>
       <c r="D36" t="str">
-        <v>Watch this and everyone will think you're a native English speaker!</v>
+        <v>How to Build Confidence &amp; Rule the World 🏆</v>
       </c>
       <c r="E36" t="str">
-        <v>Real English From Movies</v>
+        <v>Riya Upreti</v>
       </c>
       <c r="F36" t="str">
-        <v>https://www.youtube.com/watch?v=OaDhB9tgBUE</v>
+        <v>https://www.youtube.com/watch?v=G05dmSjMoCU</v>
       </c>
       <c r="G36" t="str">
         <v>No</v>
@@ -1343,16 +1343,16 @@
         <v>102</v>
       </c>
       <c r="C37" t="str">
-        <v>English</v>
+        <v>Communication Skill</v>
       </c>
       <c r="D37" t="str">
-        <v>Watch this and you'll finally speak English like in the movies! 🎬</v>
+        <v>Why your English is BETTER than you think</v>
       </c>
       <c r="E37" t="str">
-        <v>Real English From Movies</v>
+        <v>English At the Ready</v>
       </c>
       <c r="F37" t="str">
-        <v>https://www.youtube.com/watch?v=xHkHOfdp4FA</v>
+        <v>https://www.youtube.com/watch?v=qoN70QgC-xI</v>
       </c>
       <c r="G37" t="str">
         <v>No</v>
@@ -1369,16 +1369,16 @@
         <v>102</v>
       </c>
       <c r="C38" t="str">
-        <v>English</v>
+        <v>Communication Skill</v>
       </c>
       <c r="D38" t="str">
-        <v>Learn All Modal Auxiliary Verb | modal verbs in english | Modal Verbs #prienglishclasses</v>
+        <v>🔥 1000 रोज़ बोले जाने वाले Words || Most Important English Words || Daily Use Word Meaning Practice</v>
       </c>
       <c r="E38" t="str">
-        <v>PRi English Classes</v>
+        <v>English ka Gurukul</v>
       </c>
       <c r="F38" t="str">
-        <v>https://www.youtube.com/watch?v=75YfMDuRmLw</v>
+        <v>https://www.youtube.com/watch?v=qoc3d33t3sY</v>
       </c>
       <c r="G38" t="str">
         <v>No</v>
@@ -1395,16 +1395,16 @@
         <v>102</v>
       </c>
       <c r="C39" t="str">
-        <v>English</v>
+        <v>Communication Skill</v>
       </c>
       <c r="D39" t="str">
-        <v>90 days Plan to Speak English Confidently | Janhavi Panwar</v>
+        <v>How to THINK in English (and why you must)</v>
       </c>
       <c r="E39" t="str">
-        <v>Janhavi Panwar</v>
+        <v>English At the Ready</v>
       </c>
       <c r="F39" t="str">
-        <v>https://www.youtube.com/watch?v=9T54hO6h1us</v>
+        <v>https://www.youtube.com/watch?v=cohlqUEtFXs</v>
       </c>
       <c r="G39" t="str">
         <v>No</v>

</xml_diff>